<commit_message>
test(e2e-data): 修 Excel impl_code/timezone + SQL jobCode 占位对齐
ta/tb/tc Excel 包:
- impl_code:31 行 camelCase → UPPER_SNAKE
  (sftpReceiveStep → IMPORT_RECEIVE 等,对齐 BE step_registry 真实命名)
- 新增 timezone 列,15 行填 'Asia/Shanghai'(BE schema 加 NOT NULL,Excel 缺)
- tb row7 stage_code:TRANSFER → STORE(TRANSFER 不在合法 enum 内)

03-job-instance-states/seed-job-instances.sql:
- jobCode 占位 'TA_INC_ORDER_AGG' → 真实 'TA_IMPORT_ORDER'
  (依 ta 包内真实 job_code)

经 BE 修 Excel parser 后,ta/tb/tc apply 全成功(5/4/6 jobDef 入库),
SQL seed 也跑通(4 instance + 1 partition + 3 approval + 1 outbox)。
e2e 全量 381/16/5 → 95%+ 通过。

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/e2e-data/01-tenant-config-import/ta-tenant-config-package-test.xlsx
+++ b/e2e-data/01-tenant-config-import/ta-tenant-config-package-test.xlsx
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T6"/>
+  <dimension ref="A1:U6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -579,6 +579,11 @@
           <t>description</t>
         </is>
       </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>timezone</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -675,6 +680,11 @@
       <c r="T2" s="3" t="inlineStr">
         <is>
           <t>每日2点导入客户文件</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Asia/Shanghai</t>
         </is>
       </c>
     </row>
@@ -763,6 +773,11 @@
           <t>手动触发零售报表导出</t>
         </is>
       </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Asia/Shanghai</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -853,6 +868,11 @@
           <t>每5分钟分发订单</t>
         </is>
       </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Asia/Shanghai</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -935,6 +955,11 @@
           <t>每日22点结算</t>
         </is>
       </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Asia/Shanghai</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1031,6 +1056,11 @@
       <c r="T6" t="inlineStr">
         <is>
           <t>FEEDBACK 全链覆盖样本</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Asia/Shanghai</t>
         </is>
       </c>
     </row>
@@ -1745,7 +1775,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>sftpReceiveStep</t>
+          <t>IMPORT_RECEIVE</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -1799,7 +1829,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>csvParseStep</t>
+          <t>IMPORT_PARSE</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -1853,7 +1883,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>customerValidateStep</t>
+          <t>IMPORT_VALIDATE</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -1907,7 +1937,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>jdbcLoadStep</t>
+          <t>IMPORT_LOAD</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -1961,7 +1991,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>sftpReceiveStep</t>
+          <t>IMPORT_RECEIVE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -2015,7 +2045,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>orderPreprocessStep</t>
+          <t>IMPORT_PREPROCESS</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -2069,7 +2099,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>csvParseStep</t>
+          <t>IMPORT_PARSE</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -2123,7 +2153,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>orderValidateStep</t>
+          <t>IMPORT_VALIDATE</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -2177,7 +2207,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>jdbcLoadStep</t>
+          <t>IMPORT_LOAD</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -2231,7 +2261,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>orderFeedbackStep</t>
+          <t>IMPORT_FEEDBACK</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -2285,7 +2315,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>reportPrepareStep</t>
+          <t>EXPORT_PREPARE</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -2339,7 +2369,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>reportGenerateStep</t>
+          <t>EXPORT_GENERATE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -2393,7 +2423,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>reportStoreStep</t>
+          <t>EXPORT_STORE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -2447,7 +2477,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>fileRecordRegisterStep</t>
+          <t>EXPORT_REGISTER</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -2501,7 +2531,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>reportCompleteStep</t>
+          <t>EXPORT_COMPLETE</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">

</xml_diff>

<commit_message>
test(e2e): stabilize business correctness checks
</commit_message>
<xml_diff>
--- a/e2e-data/01-tenant-config-import/ta-tenant-config-package-test.xlsx
+++ b/e2e-data/01-tenant-config-import/ta-tenant-config-package-test.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="resource_queue" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="business_calendar" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="batch_window" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="job_definition" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="file_channel_config" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="file_template_config" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pipeline_definition" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pipeline_step_definition" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="workflow_definition" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="workflow_node" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="workflow_edge" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="resource_queue" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="business_calendar" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="batch_window" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="job_definition" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="file_channel_config" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="file_template_config" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="pipeline_definition" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="pipeline_step_definition" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="workflow_definition" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="workflow_node" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="workflow_edge" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -729,7 +729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -968,6 +968,114 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ta</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TA_WF_SETTLEMENT</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>START</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>开始</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>START</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ta</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TA_WF_SETTLEMENT</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>END</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>结束</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>END</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>3</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -979,7 +1087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1065,6 +1173,76 @@
       </c>
       <c r="G2" s="3" t="inlineStr"/>
       <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ta</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TA_WF_SETTLEMENT</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>START</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>NODE_IMPORT</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ta</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TA_WF_SETTLEMENT</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>NODE_EXPORT</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>END</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
@@ -1350,7 +1528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T6"/>
+  <dimension ref="A1:W6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1376,458 +1554,484 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>tenant_id</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>job_code</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>job_name</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>job_type</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>biz_type</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>queue_code</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>worker_group</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>schedule_type</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>schedule_expr</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>depends_on_job_code</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
         <is>
           <t>calendar_code</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>window_code</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>retry_policy</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>retry_max_count</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>timeout_seconds</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>shard_strategy</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>execution_mode</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>watermark_field</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
         <is>
           <t>execution_handler</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>param_schema</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>default_params</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>enabled</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>ta</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>TA_IMPORT_CUSTOMER</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>客户文件导入</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>IMPORT</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>CUSTOMER</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>ta-import-queue</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>import</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>CRON</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>0 2 * * *</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>0 0 2 * * ?</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
         <is>
           <t>default-calendar</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>always-open</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>FIXED</t>
         </is>
       </c>
-      <c r="M2" s="3" t="n">
+      <c r="N2" t="n">
         <v>3</v>
       </c>
-      <c r="N2" s="3" t="n">
+      <c r="O2" t="n">
         <v>3600</v>
       </c>
-      <c r="O2" s="3" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>
       </c>
-      <c r="P2" s="3" t="inlineStr">
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>FULL</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
         <is>
           <t>importJobHandler</t>
         </is>
       </c>
-      <c r="Q2" s="3" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="R2" s="3" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="S2" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T2" s="3" t="inlineStr">
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
         <is>
           <t>每日2点导入客户文件</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>ta</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>TA_EXPORT_REPORT</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>零售报表导出</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>EXPORT</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>REPORT</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>ta-export-queue</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>MANUAL</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr"/>
-      <c r="J3" s="3" t="inlineStr"/>
-      <c r="K3" s="3" t="inlineStr"/>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>
       </c>
-      <c r="M3" s="3" t="n">
+      <c r="N3" t="n">
         <v>0</v>
       </c>
-      <c r="N3" s="3" t="n">
+      <c r="O3" t="n">
         <v>1800</v>
       </c>
-      <c r="O3" s="3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>
       </c>
-      <c r="P3" s="3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>FULL</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
         <is>
           <t>exportJobHandler</t>
         </is>
       </c>
-      <c r="Q3" s="3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="R3" s="3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="S3" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T3" s="3" t="inlineStr">
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
         <is>
           <t>手动触发零售报表导出</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>ta</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>TA_DISPATCH_ORDER</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>订单分发</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>DISPATCH</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>ORDER</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>ta-dispatch-queue</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>dispatch</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>FIXED_RATE</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>300</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr"/>
-      <c r="K4" s="3" t="inlineStr"/>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>EXPONENTIAL</t>
         </is>
       </c>
-      <c r="M4" s="3" t="n">
+      <c r="N4" t="n">
         <v>5</v>
       </c>
-      <c r="N4" s="3" t="n">
+      <c r="O4" t="n">
         <v>600</v>
       </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>DYNAMIC</t>
         </is>
       </c>
-      <c r="P4" s="3" t="inlineStr">
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>FULL</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
         <is>
           <t>dispatchJobHandler</t>
         </is>
       </c>
-      <c r="Q4" s="3" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="R4" s="3" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="S4" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T4" s="3" t="inlineStr">
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
         <is>
           <t>每5分钟分发订单</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>ta</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>TA_WF_SETTLEMENT</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>结算工作流</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>WORKFLOW</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>SETTLE</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="3" t="inlineStr"/>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>CRON</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>0 22 * * *</t>
-        </is>
-      </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>0 0 22 * * ?</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>default-calendar</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr"/>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>
       </c>
-      <c r="M5" s="3" t="n">
+      <c r="N5" t="n">
         <v>0</v>
       </c>
-      <c r="N5" s="3" t="n">
+      <c r="O5" t="n">
         <v>7200</v>
       </c>
-      <c r="O5" s="3" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>
       </c>
-      <c r="P5" s="3" t="inlineStr"/>
-      <c r="Q5" s="3" t="inlineStr">
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>FULL</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="R5" s="3" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="S5" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T5" s="3" t="inlineStr">
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
         <is>
           <t>每日22点结算</t>
         </is>
@@ -1876,56 +2080,61 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>0 3 * * *</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
+          <t>0 0 3 * * ?</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
         <is>
           <t>default-calendar</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>always-open</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>EXPONENTIAL</t>
         </is>
       </c>
-      <c r="M6" t="n">
+      <c r="N6" t="n">
         <v>3</v>
       </c>
-      <c r="N6" t="n">
+      <c r="O6" t="n">
         <v>3600</v>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>STATIC</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>FULL</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
         <is>
           <t>orderImportHandler</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
         <is>
           <t>FEEDBACK 全链覆盖样本</t>
         </is>
@@ -2042,7 +2251,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>{"host":"sftp","port":22,"username":"ta","password":"ta_pass_123","remotePath":"/inbound"}</t>
+          <t>{"sftp_host": "sftp", "sftp_port": 22, "sftp_username": "ta", "sftp_password": "ta_pass_123", "sftp_remote_path": "/inbound"}</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -2530,12 +2739,12 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>[{"source":"id","target":"ID"}]</t>
+          <t>[{"name":"customer_no","targetColumn":"customer_no","type":"STRING","required":true},{"name":"customer_name","targetColumn":"customer_name","type":"STRING","required":true},{"name":"customer_type","targetColumn":"customer_type","type":"STRING","required":true},{"name":"certificate_no","targetColumn":"certificate_no","type":"STRING"},{"name":"mobile_no","targetColumn":"mobile_no","type":"STRING"},{"name":"email","targetColumn":"email","type":"STRING"},{"name":"status","targetColumn":"status","type":"STRING","required":true}]</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>[{"field":"id","rule":"required"}]</t>
+          <t>{"fieldRules":{"customer_no":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"},"customer_name":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"},"customer_type":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"},"status":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"}}}</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -2703,7 +2912,7 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>[{"source":"id","target":"ID"}]</t>
+          <t>[{"name":"id","sourceColumn":"id","header":"ID"},{"name":"tenant_id","sourceColumn":"tenant_id","header":"Tenant"},{"name":"customer_no","sourceColumn":"customer_no","header":"Customer No"},{"name":"customer_name","sourceColumn":"customer_name","header":"Customer Name"},{"name":"customer_type","sourceColumn":"customer_type","header":"Customer Type"},{"name":"certificate_no","sourceColumn":"certificate_no","header":"Certificate No"},{"name":"mobile_no","sourceColumn":"mobile_no","header":"Mobile"},{"name":"email","sourceColumn":"email","header":"Email"},{"name":"status","sourceColumn":"status","header":"Status"}]</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
@@ -2718,7 +2927,7 @@
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>select * from report_export</t>
+          <t>SELECT id, tenant_id, customer_no, customer_name, customer_type, certificate_no, mobile_no, email, status FROM biz.customer_account WHERE tenant_id = :tenantId AND CAST(:batchNo AS text) IS NOT NULL</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
@@ -2866,7 +3075,7 @@
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>[{"source":"id","target":"ID"}]</t>
+          <t>[{"source":"id","target":"ID","name":"id"}]</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
@@ -3039,7 +3248,7 @@
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>[{"source":"id","target":"ID"}]</t>
+          <t>[{"source":"id","target":"ID","name":"id"}]</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
@@ -3212,12 +3421,12 @@
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>[{"source":"id","target":"ID"}]</t>
+          <t>[{"name":"customer_no","targetColumn":"customer_no","type":"STRING","required":true},{"name":"customer_name","targetColumn":"customer_name","type":"STRING","required":true},{"name":"customer_type","targetColumn":"customer_type","type":"STRING","required":true},{"name":"certificate_no","targetColumn":"certificate_no","type":"STRING"},{"name":"mobile_no","targetColumn":"mobile_no","type":"STRING"},{"name":"email","targetColumn":"email","type":"STRING"},{"name":"status","targetColumn":"status","type":"STRING","required":true}]</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>[{"field":"id","rule":"required"}]</t>
+          <t>{"fieldRules":{"customer_no":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"},"customer_name":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"},"customer_type":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"},"status":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"}}}</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">
@@ -3604,7 +3813,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>sftpReceiveStep</t>
+          <t>IMPORT_RECEIVE</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -3658,7 +3867,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>csvParseStep</t>
+          <t>IMPORT_PARSE</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -3712,7 +3921,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>customerValidateStep</t>
+          <t>IMPORT_VALIDATE</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -3766,7 +3975,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>jdbcLoadStep</t>
+          <t>IMPORT_LOAD</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -3820,7 +4029,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>sftpReceiveStep</t>
+          <t>IMPORT_RECEIVE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -3874,7 +4083,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>orderPreprocessStep</t>
+          <t>IMPORT_PREPROCESS</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -3928,7 +4137,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>csvParseStep</t>
+          <t>IMPORT_PARSE</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -3982,7 +4191,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>orderValidateStep</t>
+          <t>IMPORT_VALIDATE</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -4036,7 +4245,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>jdbcLoadStep</t>
+          <t>IMPORT_LOAD</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -4090,7 +4299,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>orderFeedbackStep</t>
+          <t>IMPORT_FEEDBACK</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -4144,7 +4353,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>reportPrepareStep</t>
+          <t>EXPORT_PREPARE</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -4198,7 +4407,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>reportGenerateStep</t>
+          <t>EXPORT_GENERATE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -4252,7 +4461,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>reportStoreStep</t>
+          <t>EXPORT_STORE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -4306,7 +4515,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>fileRecordRegisterStep</t>
+          <t>EXPORT_REGISTER</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -4360,7 +4569,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>reportCompleteStep</t>
+          <t>EXPORT_COMPLETE</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">

</xml_diff>

<commit_message>
test(e2e): stabilize business correctness checks (#203)
Co-authored-by: Dengchao <tfys9544@gmail.com>
</commit_message>
<xml_diff>
--- a/e2e-data/01-tenant-config-import/ta-tenant-config-package-test.xlsx
+++ b/e2e-data/01-tenant-config-import/ta-tenant-config-package-test.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="resource_queue" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="business_calendar" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="batch_window" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="job_definition" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="file_channel_config" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="file_template_config" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pipeline_definition" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pipeline_step_definition" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="workflow_definition" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="workflow_node" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="workflow_edge" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="resource_queue" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="business_calendar" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="batch_window" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="job_definition" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="file_channel_config" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="file_template_config" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="pipeline_definition" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="pipeline_step_definition" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="workflow_definition" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="workflow_node" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="workflow_edge" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -729,7 +729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -968,6 +968,114 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ta</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TA_WF_SETTLEMENT</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>START</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>开始</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>START</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ta</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TA_WF_SETTLEMENT</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>END</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>结束</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>END</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>3</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -979,7 +1087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1065,6 +1173,76 @@
       </c>
       <c r="G2" s="3" t="inlineStr"/>
       <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ta</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TA_WF_SETTLEMENT</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>START</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>NODE_IMPORT</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ta</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TA_WF_SETTLEMENT</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>NODE_EXPORT</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>END</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
@@ -1350,7 +1528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T6"/>
+  <dimension ref="A1:W6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1376,458 +1554,484 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>tenant_id</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>job_code</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>job_name</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>job_type</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>biz_type</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>queue_code</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>worker_group</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>schedule_type</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>schedule_expr</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>depends_on_job_code</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
         <is>
           <t>calendar_code</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>window_code</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>retry_policy</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>retry_max_count</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>timeout_seconds</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>shard_strategy</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>execution_mode</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>watermark_field</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
         <is>
           <t>execution_handler</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>param_schema</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>default_params</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>enabled</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>ta</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>TA_IMPORT_CUSTOMER</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>客户文件导入</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>IMPORT</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>CUSTOMER</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>ta-import-queue</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>import</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>CRON</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>0 2 * * *</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>0 0 2 * * ?</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
         <is>
           <t>default-calendar</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>always-open</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>FIXED</t>
         </is>
       </c>
-      <c r="M2" s="3" t="n">
+      <c r="N2" t="n">
         <v>3</v>
       </c>
-      <c r="N2" s="3" t="n">
+      <c r="O2" t="n">
         <v>3600</v>
       </c>
-      <c r="O2" s="3" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>
       </c>
-      <c r="P2" s="3" t="inlineStr">
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>FULL</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
         <is>
           <t>importJobHandler</t>
         </is>
       </c>
-      <c r="Q2" s="3" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="R2" s="3" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="S2" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T2" s="3" t="inlineStr">
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
         <is>
           <t>每日2点导入客户文件</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>ta</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>TA_EXPORT_REPORT</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>零售报表导出</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>EXPORT</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>REPORT</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>ta-export-queue</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>export</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>MANUAL</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr"/>
-      <c r="J3" s="3" t="inlineStr"/>
-      <c r="K3" s="3" t="inlineStr"/>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>
       </c>
-      <c r="M3" s="3" t="n">
+      <c r="N3" t="n">
         <v>0</v>
       </c>
-      <c r="N3" s="3" t="n">
+      <c r="O3" t="n">
         <v>1800</v>
       </c>
-      <c r="O3" s="3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>
       </c>
-      <c r="P3" s="3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>FULL</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
         <is>
           <t>exportJobHandler</t>
         </is>
       </c>
-      <c r="Q3" s="3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="R3" s="3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="S3" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T3" s="3" t="inlineStr">
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
         <is>
           <t>手动触发零售报表导出</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>ta</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>TA_DISPATCH_ORDER</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>订单分发</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>DISPATCH</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>ORDER</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>ta-dispatch-queue</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>dispatch</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>FIXED_RATE</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>300</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr"/>
-      <c r="K4" s="3" t="inlineStr"/>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>EXPONENTIAL</t>
         </is>
       </c>
-      <c r="M4" s="3" t="n">
+      <c r="N4" t="n">
         <v>5</v>
       </c>
-      <c r="N4" s="3" t="n">
+      <c r="O4" t="n">
         <v>600</v>
       </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>DYNAMIC</t>
         </is>
       </c>
-      <c r="P4" s="3" t="inlineStr">
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>FULL</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
         <is>
           <t>dispatchJobHandler</t>
         </is>
       </c>
-      <c r="Q4" s="3" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="R4" s="3" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="S4" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T4" s="3" t="inlineStr">
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
         <is>
           <t>每5分钟分发订单</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>ta</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>TA_WF_SETTLEMENT</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>结算工作流</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>WORKFLOW</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>SETTLE</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="3" t="inlineStr"/>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>CRON</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>0 22 * * *</t>
-        </is>
-      </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>0 0 22 * * ?</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>default-calendar</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr"/>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>
       </c>
-      <c r="M5" s="3" t="n">
+      <c r="N5" t="n">
         <v>0</v>
       </c>
-      <c r="N5" s="3" t="n">
+      <c r="O5" t="n">
         <v>7200</v>
       </c>
-      <c r="O5" s="3" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>
       </c>
-      <c r="P5" s="3" t="inlineStr"/>
-      <c r="Q5" s="3" t="inlineStr">
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>FULL</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="R5" s="3" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="S5" s="3" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T5" s="3" t="inlineStr">
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
         <is>
           <t>每日22点结算</t>
         </is>
@@ -1876,56 +2080,61 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>0 3 * * *</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
+          <t>0 0 3 * * ?</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
         <is>
           <t>default-calendar</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>always-open</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>EXPONENTIAL</t>
         </is>
       </c>
-      <c r="M6" t="n">
+      <c r="N6" t="n">
         <v>3</v>
       </c>
-      <c r="N6" t="n">
+      <c r="O6" t="n">
         <v>3600</v>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>STATIC</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>FULL</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
         <is>
           <t>orderImportHandler</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
         <is>
           <t>FEEDBACK 全链覆盖样本</t>
         </is>
@@ -2042,7 +2251,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>{"host":"sftp","port":22,"username":"ta","password":"ta_pass_123","remotePath":"/inbound"}</t>
+          <t>{"sftp_host": "sftp", "sftp_port": 22, "sftp_username": "ta", "sftp_password": "ta_pass_123", "sftp_remote_path": "/inbound"}</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -2530,12 +2739,12 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>[{"source":"id","target":"ID"}]</t>
+          <t>[{"name":"customer_no","targetColumn":"customer_no","type":"STRING","required":true},{"name":"customer_name","targetColumn":"customer_name","type":"STRING","required":true},{"name":"customer_type","targetColumn":"customer_type","type":"STRING","required":true},{"name":"certificate_no","targetColumn":"certificate_no","type":"STRING"},{"name":"mobile_no","targetColumn":"mobile_no","type":"STRING"},{"name":"email","targetColumn":"email","type":"STRING"},{"name":"status","targetColumn":"status","type":"STRING","required":true}]</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>[{"field":"id","rule":"required"}]</t>
+          <t>{"fieldRules":{"customer_no":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"},"customer_name":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"},"customer_type":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"},"status":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"}}}</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -2703,7 +2912,7 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>[{"source":"id","target":"ID"}]</t>
+          <t>[{"name":"id","sourceColumn":"id","header":"ID"},{"name":"tenant_id","sourceColumn":"tenant_id","header":"Tenant"},{"name":"customer_no","sourceColumn":"customer_no","header":"Customer No"},{"name":"customer_name","sourceColumn":"customer_name","header":"Customer Name"},{"name":"customer_type","sourceColumn":"customer_type","header":"Customer Type"},{"name":"certificate_no","sourceColumn":"certificate_no","header":"Certificate No"},{"name":"mobile_no","sourceColumn":"mobile_no","header":"Mobile"},{"name":"email","sourceColumn":"email","header":"Email"},{"name":"status","sourceColumn":"status","header":"Status"}]</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
@@ -2718,7 +2927,7 @@
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>select * from report_export</t>
+          <t>SELECT id, tenant_id, customer_no, customer_name, customer_type, certificate_no, mobile_no, email, status FROM biz.customer_account WHERE tenant_id = :tenantId AND CAST(:batchNo AS text) IS NOT NULL</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
@@ -2866,7 +3075,7 @@
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>[{"source":"id","target":"ID"}]</t>
+          <t>[{"source":"id","target":"ID","name":"id"}]</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
@@ -3039,7 +3248,7 @@
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>[{"source":"id","target":"ID"}]</t>
+          <t>[{"source":"id","target":"ID","name":"id"}]</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
@@ -3212,12 +3421,12 @@
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>[{"source":"id","target":"ID"}]</t>
+          <t>[{"name":"customer_no","targetColumn":"customer_no","type":"STRING","required":true},{"name":"customer_name","targetColumn":"customer_name","type":"STRING","required":true},{"name":"customer_type","targetColumn":"customer_type","type":"STRING","required":true},{"name":"certificate_no","targetColumn":"certificate_no","type":"STRING"},{"name":"mobile_no","targetColumn":"mobile_no","type":"STRING"},{"name":"email","targetColumn":"email","type":"STRING"},{"name":"status","targetColumn":"status","type":"STRING","required":true}]</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>[{"field":"id","rule":"required"}]</t>
+          <t>{"fieldRules":{"customer_no":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"},"customer_name":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"},"customer_type":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"},"status":{"required":true,"errorCode":"IMPORT_VALIDATE_REQUIRED"}}}</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">
@@ -3604,7 +3813,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>sftpReceiveStep</t>
+          <t>IMPORT_RECEIVE</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -3658,7 +3867,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>csvParseStep</t>
+          <t>IMPORT_PARSE</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -3712,7 +3921,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>customerValidateStep</t>
+          <t>IMPORT_VALIDATE</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -3766,7 +3975,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>jdbcLoadStep</t>
+          <t>IMPORT_LOAD</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -3820,7 +4029,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>sftpReceiveStep</t>
+          <t>IMPORT_RECEIVE</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -3874,7 +4083,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>orderPreprocessStep</t>
+          <t>IMPORT_PREPROCESS</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -3928,7 +4137,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>csvParseStep</t>
+          <t>IMPORT_PARSE</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -3982,7 +4191,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>orderValidateStep</t>
+          <t>IMPORT_VALIDATE</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -4036,7 +4245,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>jdbcLoadStep</t>
+          <t>IMPORT_LOAD</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -4090,7 +4299,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>orderFeedbackStep</t>
+          <t>IMPORT_FEEDBACK</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -4144,7 +4353,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>reportPrepareStep</t>
+          <t>EXPORT_PREPARE</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -4198,7 +4407,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>reportGenerateStep</t>
+          <t>EXPORT_GENERATE</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -4252,7 +4461,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>reportStoreStep</t>
+          <t>EXPORT_STORE</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -4306,7 +4515,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>fileRecordRegisterStep</t>
+          <t>EXPORT_REGISTER</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -4360,7 +4569,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>reportCompleteStep</t>
+          <t>EXPORT_COMPLETE</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">

</xml_diff>